<commit_message>
add events amistoso vs Bellapampa - colectivo min40
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cantolaoaqp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB88639-5E43-4F24-8C66-6C4FA4A94ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85F4F0B-EB85-4E75-A164-F1E033AD3D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="515">
   <si>
     <t>XY</t>
   </si>
@@ -890,6 +890,681 @@
   </si>
   <si>
     <t>https://youtu.be/fE4Ma9vXx1w</t>
+  </si>
+  <si>
+    <t>20:26</t>
+  </si>
+  <si>
+    <t>20:34</t>
+  </si>
+  <si>
+    <t>20:42</t>
+  </si>
+  <si>
+    <t>89;32</t>
+  </si>
+  <si>
+    <t>20:47</t>
+  </si>
+  <si>
+    <t>20:51</t>
+  </si>
+  <si>
+    <t>20:54</t>
+  </si>
+  <si>
+    <t>36;18</t>
+  </si>
+  <si>
+    <t>20:52</t>
+  </si>
+  <si>
+    <t>20:56</t>
+  </si>
+  <si>
+    <t>21:00</t>
+  </si>
+  <si>
+    <t>29;40</t>
+  </si>
+  <si>
+    <t>20:59</t>
+  </si>
+  <si>
+    <t>21:02</t>
+  </si>
+  <si>
+    <t>21:05</t>
+  </si>
+  <si>
+    <t>64;39</t>
+  </si>
+  <si>
+    <t>21:04</t>
+  </si>
+  <si>
+    <t>21:13</t>
+  </si>
+  <si>
+    <t>21:22</t>
+  </si>
+  <si>
+    <t>55;51</t>
+  </si>
+  <si>
+    <t>21:26</t>
+  </si>
+  <si>
+    <t>21:38</t>
+  </si>
+  <si>
+    <t>21:50</t>
+  </si>
+  <si>
+    <t>74;56</t>
+  </si>
+  <si>
+    <t>21:49</t>
+  </si>
+  <si>
+    <t>21:55</t>
+  </si>
+  <si>
+    <t>22:02</t>
+  </si>
+  <si>
+    <t>18;12</t>
+  </si>
+  <si>
+    <t>22:10</t>
+  </si>
+  <si>
+    <t>22:19</t>
+  </si>
+  <si>
+    <t>56;32</t>
+  </si>
+  <si>
+    <t>22:18</t>
+  </si>
+  <si>
+    <t>22:22</t>
+  </si>
+  <si>
+    <t>22:27</t>
+  </si>
+  <si>
+    <t>30;70</t>
+  </si>
+  <si>
+    <t>22:37</t>
+  </si>
+  <si>
+    <t>22:45</t>
+  </si>
+  <si>
+    <t>22:52</t>
+  </si>
+  <si>
+    <t>21;75</t>
+  </si>
+  <si>
+    <t>22:51</t>
+  </si>
+  <si>
+    <t>23:00</t>
+  </si>
+  <si>
+    <t>23:08</t>
+  </si>
+  <si>
+    <t>65;13</t>
+  </si>
+  <si>
+    <t>23:11</t>
+  </si>
+  <si>
+    <t>23:16</t>
+  </si>
+  <si>
+    <t>23:21</t>
+  </si>
+  <si>
+    <t>69;89</t>
+  </si>
+  <si>
+    <t>23:29</t>
+  </si>
+  <si>
+    <t>23:34</t>
+  </si>
+  <si>
+    <t>23:40</t>
+  </si>
+  <si>
+    <t>89;66</t>
+  </si>
+  <si>
+    <t>23:59</t>
+  </si>
+  <si>
+    <t>24:02</t>
+  </si>
+  <si>
+    <t>24:05</t>
+  </si>
+  <si>
+    <t>75;82</t>
+  </si>
+  <si>
+    <t>24:04</t>
+  </si>
+  <si>
+    <t>24:10</t>
+  </si>
+  <si>
+    <t>24:15</t>
+  </si>
+  <si>
+    <t>64;44</t>
+  </si>
+  <si>
+    <t>24:32</t>
+  </si>
+  <si>
+    <t>24:36</t>
+  </si>
+  <si>
+    <t>24:41</t>
+  </si>
+  <si>
+    <t>94;46</t>
+  </si>
+  <si>
+    <t>24:38</t>
+  </si>
+  <si>
+    <t>24:46</t>
+  </si>
+  <si>
+    <t>24:54</t>
+  </si>
+  <si>
+    <t>64;28</t>
+  </si>
+  <si>
+    <t>25:12</t>
+  </si>
+  <si>
+    <t>25:21</t>
+  </si>
+  <si>
+    <t>25:30</t>
+  </si>
+  <si>
+    <t>90;87</t>
+  </si>
+  <si>
+    <t>25:35</t>
+  </si>
+  <si>
+    <t>25:40</t>
+  </si>
+  <si>
+    <t>25:45</t>
+  </si>
+  <si>
+    <t>14;53</t>
+  </si>
+  <si>
+    <t>25:51</t>
+  </si>
+  <si>
+    <t>26:04</t>
+  </si>
+  <si>
+    <t>26:17</t>
+  </si>
+  <si>
+    <t>28;8</t>
+  </si>
+  <si>
+    <t>27:05</t>
+  </si>
+  <si>
+    <t>27:14</t>
+  </si>
+  <si>
+    <t>27:24</t>
+  </si>
+  <si>
+    <t>54;47</t>
+  </si>
+  <si>
+    <t>27:43</t>
+  </si>
+  <si>
+    <t>27:50</t>
+  </si>
+  <si>
+    <t>27:57</t>
+  </si>
+  <si>
+    <t>65;9</t>
+  </si>
+  <si>
+    <t>28:00</t>
+  </si>
+  <si>
+    <t>28:06</t>
+  </si>
+  <si>
+    <t>28:12</t>
+  </si>
+  <si>
+    <t>35;51</t>
+  </si>
+  <si>
+    <t>28:17</t>
+  </si>
+  <si>
+    <t>28:21</t>
+  </si>
+  <si>
+    <t>55;90</t>
+  </si>
+  <si>
+    <t>28:22</t>
+  </si>
+  <si>
+    <t>28:26</t>
+  </si>
+  <si>
+    <t>28:30</t>
+  </si>
+  <si>
+    <t>66;39</t>
+  </si>
+  <si>
+    <t>28:33</t>
+  </si>
+  <si>
+    <t>28:41</t>
+  </si>
+  <si>
+    <t>28:49</t>
+  </si>
+  <si>
+    <t>89;71</t>
+  </si>
+  <si>
+    <t>28:47</t>
+  </si>
+  <si>
+    <t>28:51</t>
+  </si>
+  <si>
+    <t>28:54</t>
+  </si>
+  <si>
+    <t>76;52</t>
+  </si>
+  <si>
+    <t>28:52</t>
+  </si>
+  <si>
+    <t>28:57</t>
+  </si>
+  <si>
+    <t>29:01</t>
+  </si>
+  <si>
+    <t>72;77</t>
+  </si>
+  <si>
+    <t>29:18</t>
+  </si>
+  <si>
+    <t>29:27</t>
+  </si>
+  <si>
+    <t>72;17</t>
+  </si>
+  <si>
+    <t>29:22</t>
+  </si>
+  <si>
+    <t>29:28</t>
+  </si>
+  <si>
+    <t>29:33</t>
+  </si>
+  <si>
+    <t>35;69</t>
+  </si>
+  <si>
+    <t>29:30</t>
+  </si>
+  <si>
+    <t>29:34</t>
+  </si>
+  <si>
+    <t>29:37</t>
+  </si>
+  <si>
+    <t>88;91</t>
+  </si>
+  <si>
+    <t>29:45</t>
+  </si>
+  <si>
+    <t>30:00</t>
+  </si>
+  <si>
+    <t>30:16</t>
+  </si>
+  <si>
+    <t>95;86</t>
+  </si>
+  <si>
+    <t>30:37</t>
+  </si>
+  <si>
+    <t>31:01</t>
+  </si>
+  <si>
+    <t>31:26</t>
+  </si>
+  <si>
+    <t>27;85</t>
+  </si>
+  <si>
+    <t>Ocasión rival</t>
+  </si>
+  <si>
+    <t>31:54</t>
+  </si>
+  <si>
+    <t>32:05</t>
+  </si>
+  <si>
+    <t>32:16</t>
+  </si>
+  <si>
+    <t>75;91</t>
+  </si>
+  <si>
+    <t>32:15</t>
+  </si>
+  <si>
+    <t>32:23</t>
+  </si>
+  <si>
+    <t>32:30</t>
+  </si>
+  <si>
+    <t>30;59</t>
+  </si>
+  <si>
+    <t>32:45</t>
+  </si>
+  <si>
+    <t>32:57</t>
+  </si>
+  <si>
+    <t>33:09</t>
+  </si>
+  <si>
+    <t>79;51</t>
+  </si>
+  <si>
+    <t>33:29</t>
+  </si>
+  <si>
+    <t>33:32</t>
+  </si>
+  <si>
+    <t>33:35</t>
+  </si>
+  <si>
+    <t>47;46</t>
+  </si>
+  <si>
+    <t>33:34</t>
+  </si>
+  <si>
+    <t>33:39</t>
+  </si>
+  <si>
+    <t>33:44</t>
+  </si>
+  <si>
+    <t>55;23</t>
+  </si>
+  <si>
+    <t>33:43</t>
+  </si>
+  <si>
+    <t>33:52</t>
+  </si>
+  <si>
+    <t>34:01</t>
+  </si>
+  <si>
+    <t>34:35</t>
+  </si>
+  <si>
+    <t>34:54</t>
+  </si>
+  <si>
+    <t>35:12</t>
+  </si>
+  <si>
+    <t>40;14</t>
+  </si>
+  <si>
+    <t>35:20</t>
+  </si>
+  <si>
+    <t>35:27</t>
+  </si>
+  <si>
+    <t>35:34</t>
+  </si>
+  <si>
+    <t>7;87</t>
+  </si>
+  <si>
+    <t>35:46</t>
+  </si>
+  <si>
+    <t>35:49</t>
+  </si>
+  <si>
+    <t>35:52</t>
+  </si>
+  <si>
+    <t>41;94</t>
+  </si>
+  <si>
+    <t>36:06</t>
+  </si>
+  <si>
+    <t>36:15</t>
+  </si>
+  <si>
+    <t>36:23</t>
+  </si>
+  <si>
+    <t>36;22</t>
+  </si>
+  <si>
+    <t>37:01</t>
+  </si>
+  <si>
+    <t>37:04</t>
+  </si>
+  <si>
+    <t>37:07</t>
+  </si>
+  <si>
+    <t>19;72</t>
+  </si>
+  <si>
+    <t>37:13</t>
+  </si>
+  <si>
+    <t>37:18</t>
+  </si>
+  <si>
+    <t>37:33</t>
+  </si>
+  <si>
+    <t>37:38</t>
+  </si>
+  <si>
+    <t>37:43</t>
+  </si>
+  <si>
+    <t>41;77</t>
+  </si>
+  <si>
+    <t>37:41</t>
+  </si>
+  <si>
+    <t>37:45</t>
+  </si>
+  <si>
+    <t>37:49</t>
+  </si>
+  <si>
+    <t>55;79</t>
+  </si>
+  <si>
+    <t>37:47</t>
+  </si>
+  <si>
+    <t>37:51</t>
+  </si>
+  <si>
+    <t>37:55</t>
+  </si>
+  <si>
+    <t>51;23</t>
+  </si>
+  <si>
+    <t>38:29</t>
+  </si>
+  <si>
+    <t>38:33</t>
+  </si>
+  <si>
+    <t>38:37</t>
+  </si>
+  <si>
+    <t>55;10</t>
+  </si>
+  <si>
+    <t>38:44</t>
+  </si>
+  <si>
+    <t>38:50</t>
+  </si>
+  <si>
+    <t>38:56</t>
+  </si>
+  <si>
+    <t>91;47</t>
+  </si>
+  <si>
+    <t>38:57</t>
+  </si>
+  <si>
+    <t>39:01</t>
+  </si>
+  <si>
+    <t>39:04</t>
+  </si>
+  <si>
+    <t>14;6</t>
+  </si>
+  <si>
+    <t>39:12</t>
+  </si>
+  <si>
+    <t>39:15</t>
+  </si>
+  <si>
+    <t>39:18</t>
+  </si>
+  <si>
+    <t>60;17</t>
+  </si>
+  <si>
+    <t>39:23</t>
+  </si>
+  <si>
+    <t>39:28</t>
+  </si>
+  <si>
+    <t>65;26</t>
+  </si>
+  <si>
+    <t>39:34</t>
+  </si>
+  <si>
+    <t>39:41</t>
+  </si>
+  <si>
+    <t>55;19</t>
+  </si>
+  <si>
+    <t>39:38</t>
+  </si>
+  <si>
+    <t>39:46</t>
+  </si>
+  <si>
+    <t>39:54</t>
+  </si>
+  <si>
+    <t>41;44</t>
+  </si>
+  <si>
+    <t>39:51</t>
+  </si>
+  <si>
+    <t>39:58</t>
+  </si>
+  <si>
+    <t>40:05</t>
+  </si>
+  <si>
+    <t>31;14</t>
+  </si>
+  <si>
+    <t>40:31</t>
+  </si>
+  <si>
+    <t>40:35</t>
+  </si>
+  <si>
+    <t>40:39</t>
+  </si>
+  <si>
+    <t>3;9</t>
+  </si>
+  <si>
+    <t>Corner</t>
+  </si>
+  <si>
+    <t>GOL</t>
+  </si>
+  <si>
+    <t>2T</t>
+  </si>
+  <si>
+    <t>True</t>
   </si>
 </sst>
 </file>
@@ -972,8 +1647,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}" name="Tabla1" displayName="Tabla1" ref="A1:O67" totalsRowShown="0">
-  <autoFilter ref="A1:O67" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}" name="Tabla1" displayName="Tabla1" ref="A1:O124" totalsRowShown="0">
+  <autoFilter ref="A1:O124" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{45CCCD5A-AFCF-487D-ADA1-0BFBB6505772}" name="Event"/>
     <tableColumn id="2" xr3:uid="{4A939A0F-B787-4665-B94F-35DE80E0B243}" name="start_time" dataDxfId="2"/>
@@ -1282,7 +1957,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77939FC4-FC73-4262-977F-310955BE7B1D}">
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O124"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5703125" customWidth="1"/>
@@ -3896,6 +4571,2199 @@
         <v>55</v>
       </c>
     </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>14</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="E68" t="s">
+        <v>293</v>
+      </c>
+      <c r="F68" t="s">
+        <v>42</v>
+      </c>
+      <c r="G68" t="s">
+        <v>287</v>
+      </c>
+      <c r="H68" t="s">
+        <v>288</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J68" s="1"/>
+      <c r="M68" t="s">
+        <v>7</v>
+      </c>
+      <c r="N68" t="s">
+        <v>50</v>
+      </c>
+      <c r="O68" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>122</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="E69" t="s">
+        <v>297</v>
+      </c>
+      <c r="F69" t="s">
+        <v>20</v>
+      </c>
+      <c r="G69" t="s">
+        <v>46</v>
+      </c>
+      <c r="H69" t="s">
+        <v>288</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J69" s="1"/>
+      <c r="M69" t="s">
+        <v>7</v>
+      </c>
+      <c r="N69" t="s">
+        <v>50</v>
+      </c>
+      <c r="O69" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>127</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="E70" t="s">
+        <v>301</v>
+      </c>
+      <c r="F70" t="s">
+        <v>43</v>
+      </c>
+      <c r="G70" t="s">
+        <v>47</v>
+      </c>
+      <c r="H70" t="s">
+        <v>288</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J70" s="1"/>
+      <c r="M70" t="s">
+        <v>7</v>
+      </c>
+      <c r="N70" t="s">
+        <v>50</v>
+      </c>
+      <c r="O70" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>122</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="E71" t="s">
+        <v>305</v>
+      </c>
+      <c r="F71" t="s">
+        <v>20</v>
+      </c>
+      <c r="G71" t="s">
+        <v>46</v>
+      </c>
+      <c r="H71" t="s">
+        <v>288</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J71" s="1"/>
+      <c r="M71" t="s">
+        <v>7</v>
+      </c>
+      <c r="N71" t="s">
+        <v>50</v>
+      </c>
+      <c r="O71" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>127</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="E72" t="s">
+        <v>309</v>
+      </c>
+      <c r="F72" t="s">
+        <v>43</v>
+      </c>
+      <c r="G72" t="s">
+        <v>45</v>
+      </c>
+      <c r="H72" t="s">
+        <v>288</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J72" s="1"/>
+      <c r="M72" t="s">
+        <v>7</v>
+      </c>
+      <c r="N72" t="s">
+        <v>50</v>
+      </c>
+      <c r="O72" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>122</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="E73" t="s">
+        <v>313</v>
+      </c>
+      <c r="F73" t="s">
+        <v>20</v>
+      </c>
+      <c r="G73" t="s">
+        <v>287</v>
+      </c>
+      <c r="H73" t="s">
+        <v>288</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J73" s="1"/>
+      <c r="M73" t="s">
+        <v>7</v>
+      </c>
+      <c r="N73" t="s">
+        <v>50</v>
+      </c>
+      <c r="O73" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>127</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="E74" t="s">
+        <v>317</v>
+      </c>
+      <c r="F74" t="s">
+        <v>1</v>
+      </c>
+      <c r="G74" t="s">
+        <v>47</v>
+      </c>
+      <c r="H74" t="s">
+        <v>288</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J74" s="1"/>
+      <c r="M74" t="s">
+        <v>7</v>
+      </c>
+      <c r="N74" t="s">
+        <v>50</v>
+      </c>
+      <c r="O74" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>122</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="E75" t="s">
+        <v>320</v>
+      </c>
+      <c r="F75" t="s">
+        <v>20</v>
+      </c>
+      <c r="G75" t="s">
+        <v>46</v>
+      </c>
+      <c r="H75" t="s">
+        <v>288</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J75" s="1"/>
+      <c r="M75" t="s">
+        <v>7</v>
+      </c>
+      <c r="N75" t="s">
+        <v>50</v>
+      </c>
+      <c r="O75" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>127</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E76" t="s">
+        <v>324</v>
+      </c>
+      <c r="F76" t="s">
+        <v>43</v>
+      </c>
+      <c r="G76" t="s">
+        <v>45</v>
+      </c>
+      <c r="H76" t="s">
+        <v>288</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J76" s="1"/>
+      <c r="M76" t="s">
+        <v>7</v>
+      </c>
+      <c r="N76" t="s">
+        <v>50</v>
+      </c>
+      <c r="O76" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>2</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="E77" t="s">
+        <v>328</v>
+      </c>
+      <c r="F77" t="s">
+        <v>3</v>
+      </c>
+      <c r="G77" t="s">
+        <v>47</v>
+      </c>
+      <c r="H77" t="s">
+        <v>288</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J77" s="1"/>
+      <c r="M77" t="s">
+        <v>7</v>
+      </c>
+      <c r="N77" t="s">
+        <v>50</v>
+      </c>
+      <c r="O77" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>122</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E78" t="s">
+        <v>332</v>
+      </c>
+      <c r="F78" t="s">
+        <v>20</v>
+      </c>
+      <c r="G78" t="s">
+        <v>48</v>
+      </c>
+      <c r="H78" t="s">
+        <v>288</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J78" s="1"/>
+      <c r="M78" t="s">
+        <v>7</v>
+      </c>
+      <c r="N78" t="s">
+        <v>50</v>
+      </c>
+      <c r="O78" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>14</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E79" t="s">
+        <v>336</v>
+      </c>
+      <c r="F79" t="s">
+        <v>42</v>
+      </c>
+      <c r="G79" t="s">
+        <v>48</v>
+      </c>
+      <c r="H79" t="s">
+        <v>288</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J79" s="1"/>
+      <c r="M79" t="s">
+        <v>7</v>
+      </c>
+      <c r="N79" t="s">
+        <v>50</v>
+      </c>
+      <c r="O79" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>14</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="E80" t="s">
+        <v>340</v>
+      </c>
+      <c r="F80" t="s">
+        <v>20</v>
+      </c>
+      <c r="G80" t="s">
+        <v>48</v>
+      </c>
+      <c r="H80" t="s">
+        <v>288</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J80" s="1"/>
+      <c r="M80" t="s">
+        <v>7</v>
+      </c>
+      <c r="N80" t="s">
+        <v>50</v>
+      </c>
+      <c r="O80" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>27</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="E81" t="s">
+        <v>344</v>
+      </c>
+      <c r="F81" t="s">
+        <v>15</v>
+      </c>
+      <c r="H81" t="s">
+        <v>288</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J81" s="1"/>
+      <c r="M81" t="s">
+        <v>7</v>
+      </c>
+      <c r="N81" t="s">
+        <v>50</v>
+      </c>
+      <c r="O81" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>127</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="E82" t="s">
+        <v>348</v>
+      </c>
+      <c r="F82" t="s">
+        <v>45</v>
+      </c>
+      <c r="G82" t="s">
+        <v>43</v>
+      </c>
+      <c r="H82" t="s">
+        <v>288</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J82" s="1"/>
+      <c r="M82" t="s">
+        <v>7</v>
+      </c>
+      <c r="N82" t="s">
+        <v>50</v>
+      </c>
+      <c r="O82" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>14</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="E83" t="s">
+        <v>352</v>
+      </c>
+      <c r="G83" t="s">
+        <v>46</v>
+      </c>
+      <c r="H83" t="s">
+        <v>288</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J83" s="1"/>
+      <c r="M83" t="s">
+        <v>7</v>
+      </c>
+      <c r="N83" t="s">
+        <v>50</v>
+      </c>
+      <c r="O83" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>127</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E84" t="s">
+        <v>356</v>
+      </c>
+      <c r="F84" t="s">
+        <v>43</v>
+      </c>
+      <c r="G84" t="s">
+        <v>49</v>
+      </c>
+      <c r="H84" t="s">
+        <v>288</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J84" s="1"/>
+      <c r="M84" t="s">
+        <v>7</v>
+      </c>
+      <c r="N84" t="s">
+        <v>50</v>
+      </c>
+      <c r="O84" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>14</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="E85" t="s">
+        <v>360</v>
+      </c>
+      <c r="F85" t="s">
+        <v>20</v>
+      </c>
+      <c r="G85" t="s">
+        <v>287</v>
+      </c>
+      <c r="H85" t="s">
+        <v>288</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J85" s="1"/>
+      <c r="M85" t="s">
+        <v>7</v>
+      </c>
+      <c r="N85" t="s">
+        <v>50</v>
+      </c>
+      <c r="O85" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>2</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>364</v>
+      </c>
+      <c r="F86" t="s">
+        <v>17</v>
+      </c>
+      <c r="G86" t="s">
+        <v>44</v>
+      </c>
+      <c r="H86" t="s">
+        <v>288</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J86" s="1"/>
+      <c r="M86" t="s">
+        <v>7</v>
+      </c>
+      <c r="N86" t="s">
+        <v>50</v>
+      </c>
+      <c r="O86" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>2</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="E87" t="s">
+        <v>368</v>
+      </c>
+      <c r="F87" t="s">
+        <v>18</v>
+      </c>
+      <c r="G87" t="s">
+        <v>49</v>
+      </c>
+      <c r="H87" t="s">
+        <v>288</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J87" s="1"/>
+      <c r="M87" t="s">
+        <v>7</v>
+      </c>
+      <c r="N87" t="s">
+        <v>50</v>
+      </c>
+      <c r="O87" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>14</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="E88" t="s">
+        <v>372</v>
+      </c>
+      <c r="F88" t="s">
+        <v>42</v>
+      </c>
+      <c r="G88" t="s">
+        <v>48</v>
+      </c>
+      <c r="H88" t="s">
+        <v>288</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J88" s="1"/>
+      <c r="M88" t="s">
+        <v>7</v>
+      </c>
+      <c r="N88" t="s">
+        <v>50</v>
+      </c>
+      <c r="O88" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>14</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="E89" t="s">
+        <v>376</v>
+      </c>
+      <c r="F89" t="s">
+        <v>42</v>
+      </c>
+      <c r="G89" t="s">
+        <v>46</v>
+      </c>
+      <c r="H89" t="s">
+        <v>288</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J89" s="1"/>
+      <c r="M89" t="s">
+        <v>7</v>
+      </c>
+      <c r="N89" t="s">
+        <v>50</v>
+      </c>
+      <c r="O89" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>127</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="E90" t="s">
+        <v>380</v>
+      </c>
+      <c r="F90" t="s">
+        <v>43</v>
+      </c>
+      <c r="G90" t="s">
+        <v>47</v>
+      </c>
+      <c r="H90" t="s">
+        <v>288</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J90" s="1"/>
+      <c r="M90" t="s">
+        <v>7</v>
+      </c>
+      <c r="N90" t="s">
+        <v>50</v>
+      </c>
+      <c r="O90" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>127</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E91" t="s">
+        <v>383</v>
+      </c>
+      <c r="F91" t="s">
+        <v>43</v>
+      </c>
+      <c r="G91" t="s">
+        <v>47</v>
+      </c>
+      <c r="H91" t="s">
+        <v>288</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J91" s="1"/>
+      <c r="M91" t="s">
+        <v>7</v>
+      </c>
+      <c r="N91" t="s">
+        <v>50</v>
+      </c>
+      <c r="O91" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>127</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E92" t="s">
+        <v>387</v>
+      </c>
+      <c r="F92" t="s">
+        <v>43</v>
+      </c>
+      <c r="G92" t="s">
+        <v>47</v>
+      </c>
+      <c r="H92" t="s">
+        <v>288</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J92" s="1"/>
+      <c r="M92" t="s">
+        <v>7</v>
+      </c>
+      <c r="N92" t="s">
+        <v>50</v>
+      </c>
+      <c r="O92" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>14</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="E93" t="s">
+        <v>391</v>
+      </c>
+      <c r="F93" t="s">
+        <v>42</v>
+      </c>
+      <c r="G93" t="s">
+        <v>46</v>
+      </c>
+      <c r="H93" t="s">
+        <v>288</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J93" s="1"/>
+      <c r="M93" t="s">
+        <v>7</v>
+      </c>
+      <c r="N93" t="s">
+        <v>50</v>
+      </c>
+      <c r="O93" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>127</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="E94" t="s">
+        <v>395</v>
+      </c>
+      <c r="F94" t="s">
+        <v>43</v>
+      </c>
+      <c r="G94" t="s">
+        <v>47</v>
+      </c>
+      <c r="H94" t="s">
+        <v>288</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J94" s="1"/>
+      <c r="M94" t="s">
+        <v>7</v>
+      </c>
+      <c r="N94" t="s">
+        <v>50</v>
+      </c>
+      <c r="O94" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>122</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="E95" t="s">
+        <v>399</v>
+      </c>
+      <c r="F95" t="s">
+        <v>20</v>
+      </c>
+      <c r="G95" t="s">
+        <v>46</v>
+      </c>
+      <c r="H95" t="s">
+        <v>288</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J95" s="1"/>
+      <c r="M95" t="s">
+        <v>7</v>
+      </c>
+      <c r="N95" t="s">
+        <v>50</v>
+      </c>
+      <c r="O95" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>127</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="E96" t="s">
+        <v>402</v>
+      </c>
+      <c r="F96" t="s">
+        <v>1</v>
+      </c>
+      <c r="G96" t="s">
+        <v>44</v>
+      </c>
+      <c r="H96" t="s">
+        <v>288</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J96" s="1"/>
+      <c r="M96" t="s">
+        <v>7</v>
+      </c>
+      <c r="N96" t="s">
+        <v>50</v>
+      </c>
+      <c r="O96" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="E97" t="s">
+        <v>406</v>
+      </c>
+      <c r="F97" t="s">
+        <v>3</v>
+      </c>
+      <c r="G97" t="s">
+        <v>47</v>
+      </c>
+      <c r="H97" t="s">
+        <v>288</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J97" s="1"/>
+      <c r="M97" t="s">
+        <v>7</v>
+      </c>
+      <c r="N97" t="s">
+        <v>50</v>
+      </c>
+      <c r="O97" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>122</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="E98" t="s">
+        <v>410</v>
+      </c>
+      <c r="F98" t="s">
+        <v>20</v>
+      </c>
+      <c r="G98" t="s">
+        <v>48</v>
+      </c>
+      <c r="H98" t="s">
+        <v>288</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J98" s="1"/>
+      <c r="M98" t="s">
+        <v>7</v>
+      </c>
+      <c r="N98" t="s">
+        <v>50</v>
+      </c>
+      <c r="O98" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>14</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E99" t="s">
+        <v>414</v>
+      </c>
+      <c r="F99" t="s">
+        <v>42</v>
+      </c>
+      <c r="H99" t="s">
+        <v>288</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J99" s="1"/>
+      <c r="M99" t="s">
+        <v>7</v>
+      </c>
+      <c r="N99" t="s">
+        <v>50</v>
+      </c>
+      <c r="O99" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>14</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E100" t="s">
+        <v>418</v>
+      </c>
+      <c r="F100" t="s">
+        <v>42</v>
+      </c>
+      <c r="G100" t="s">
+        <v>419</v>
+      </c>
+      <c r="H100" t="s">
+        <v>288</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J100" s="1"/>
+      <c r="L100" t="s">
+        <v>512</v>
+      </c>
+      <c r="M100" t="s">
+        <v>513</v>
+      </c>
+      <c r="N100" t="s">
+        <v>514</v>
+      </c>
+      <c r="O100" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="E101" t="s">
+        <v>423</v>
+      </c>
+      <c r="F101" t="s">
+        <v>17</v>
+      </c>
+      <c r="G101" t="s">
+        <v>45</v>
+      </c>
+      <c r="H101" t="s">
+        <v>288</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J101" s="1"/>
+      <c r="M101" t="s">
+        <v>513</v>
+      </c>
+      <c r="N101" t="s">
+        <v>514</v>
+      </c>
+      <c r="O101" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>122</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="E102" t="s">
+        <v>427</v>
+      </c>
+      <c r="F102" t="s">
+        <v>21</v>
+      </c>
+      <c r="G102" t="s">
+        <v>287</v>
+      </c>
+      <c r="H102" t="s">
+        <v>288</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J102" s="1"/>
+      <c r="M102" t="s">
+        <v>513</v>
+      </c>
+      <c r="N102" t="s">
+        <v>514</v>
+      </c>
+      <c r="O102" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>2</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="E103" t="s">
+        <v>431</v>
+      </c>
+      <c r="F103" t="s">
+        <v>17</v>
+      </c>
+      <c r="G103" t="s">
+        <v>49</v>
+      </c>
+      <c r="H103" t="s">
+        <v>288</v>
+      </c>
+      <c r="I103" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J103" s="1"/>
+      <c r="M103" t="s">
+        <v>513</v>
+      </c>
+      <c r="N103" t="s">
+        <v>514</v>
+      </c>
+      <c r="O103" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>14</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="E104" t="s">
+        <v>435</v>
+      </c>
+      <c r="G104" t="s">
+        <v>46</v>
+      </c>
+      <c r="H104" t="s">
+        <v>288</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J104" s="1"/>
+      <c r="M104" t="s">
+        <v>513</v>
+      </c>
+      <c r="N104" t="s">
+        <v>514</v>
+      </c>
+      <c r="O104" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>127</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="E105" t="s">
+        <v>439</v>
+      </c>
+      <c r="F105" t="s">
+        <v>43</v>
+      </c>
+      <c r="G105" t="s">
+        <v>45</v>
+      </c>
+      <c r="H105" t="s">
+        <v>288</v>
+      </c>
+      <c r="I105" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J105" s="1"/>
+      <c r="M105" t="s">
+        <v>513</v>
+      </c>
+      <c r="N105" t="s">
+        <v>514</v>
+      </c>
+      <c r="O105" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>122</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="F106" t="s">
+        <v>20</v>
+      </c>
+      <c r="G106" t="s">
+        <v>287</v>
+      </c>
+      <c r="H106" t="s">
+        <v>288</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J106" s="1"/>
+      <c r="M106" t="s">
+        <v>513</v>
+      </c>
+      <c r="N106" t="s">
+        <v>514</v>
+      </c>
+      <c r="O106" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>2</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="E107" t="s">
+        <v>446</v>
+      </c>
+      <c r="F107" t="s">
+        <v>17</v>
+      </c>
+      <c r="G107" t="s">
+        <v>45</v>
+      </c>
+      <c r="H107" t="s">
+        <v>288</v>
+      </c>
+      <c r="I107" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J107" s="1"/>
+      <c r="M107" t="s">
+        <v>513</v>
+      </c>
+      <c r="N107" t="s">
+        <v>514</v>
+      </c>
+      <c r="O107" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>14</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E108" t="s">
+        <v>450</v>
+      </c>
+      <c r="F108" t="s">
+        <v>20</v>
+      </c>
+      <c r="G108" t="s">
+        <v>48</v>
+      </c>
+      <c r="H108" t="s">
+        <v>288</v>
+      </c>
+      <c r="I108" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J108" s="1"/>
+      <c r="M108" t="s">
+        <v>513</v>
+      </c>
+      <c r="N108" t="s">
+        <v>514</v>
+      </c>
+      <c r="O108" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>14</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="E109" t="s">
+        <v>454</v>
+      </c>
+      <c r="G109" t="s">
+        <v>46</v>
+      </c>
+      <c r="H109" t="s">
+        <v>288</v>
+      </c>
+      <c r="I109" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J109" s="1"/>
+      <c r="M109" t="s">
+        <v>513</v>
+      </c>
+      <c r="N109" t="s">
+        <v>514</v>
+      </c>
+      <c r="O109" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="E110" t="s">
+        <v>458</v>
+      </c>
+      <c r="F110" t="s">
+        <v>17</v>
+      </c>
+      <c r="G110" t="s">
+        <v>45</v>
+      </c>
+      <c r="H110" t="s">
+        <v>288</v>
+      </c>
+      <c r="I110" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J110" s="1"/>
+      <c r="M110" t="s">
+        <v>513</v>
+      </c>
+      <c r="N110" t="s">
+        <v>514</v>
+      </c>
+      <c r="O110" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>32</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="E111" t="s">
+        <v>462</v>
+      </c>
+      <c r="F111" t="s">
+        <v>4</v>
+      </c>
+      <c r="H111" t="s">
+        <v>288</v>
+      </c>
+      <c r="I111" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J111" s="1"/>
+      <c r="M111" t="s">
+        <v>513</v>
+      </c>
+      <c r="N111" t="s">
+        <v>514</v>
+      </c>
+      <c r="O111" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>127</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="F112" t="s">
+        <v>43</v>
+      </c>
+      <c r="G112" t="s">
+        <v>49</v>
+      </c>
+      <c r="H112" t="s">
+        <v>288</v>
+      </c>
+      <c r="I112" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J112" s="1"/>
+      <c r="M112" t="s">
+        <v>513</v>
+      </c>
+      <c r="N112" t="s">
+        <v>514</v>
+      </c>
+      <c r="O112" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>14</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="E113" t="s">
+        <v>468</v>
+      </c>
+      <c r="F113" t="s">
+        <v>20</v>
+      </c>
+      <c r="G113" t="s">
+        <v>46</v>
+      </c>
+      <c r="H113" t="s">
+        <v>288</v>
+      </c>
+      <c r="I113" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J113" s="1"/>
+      <c r="M113" t="s">
+        <v>513</v>
+      </c>
+      <c r="N113" t="s">
+        <v>514</v>
+      </c>
+      <c r="O113" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>127</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="E114" t="s">
+        <v>472</v>
+      </c>
+      <c r="F114" t="s">
+        <v>43</v>
+      </c>
+      <c r="G114" t="s">
+        <v>47</v>
+      </c>
+      <c r="H114" t="s">
+        <v>288</v>
+      </c>
+      <c r="I114" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J114" s="1"/>
+      <c r="M114" t="s">
+        <v>513</v>
+      </c>
+      <c r="N114" t="s">
+        <v>514</v>
+      </c>
+      <c r="O114" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>122</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="E115" t="s">
+        <v>476</v>
+      </c>
+      <c r="F115" t="s">
+        <v>20</v>
+      </c>
+      <c r="G115" t="s">
+        <v>48</v>
+      </c>
+      <c r="H115" t="s">
+        <v>288</v>
+      </c>
+      <c r="I115" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J115" s="1"/>
+      <c r="M115" t="s">
+        <v>513</v>
+      </c>
+      <c r="N115" t="s">
+        <v>514</v>
+      </c>
+      <c r="O115" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>27</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="E116" t="s">
+        <v>480</v>
+      </c>
+      <c r="F116" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" t="s">
+        <v>288</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J116" s="1"/>
+      <c r="M116" t="s">
+        <v>513</v>
+      </c>
+      <c r="N116" t="s">
+        <v>514</v>
+      </c>
+      <c r="O116" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>2</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="E117" t="s">
+        <v>484</v>
+      </c>
+      <c r="F117" t="s">
+        <v>3</v>
+      </c>
+      <c r="G117" t="s">
+        <v>45</v>
+      </c>
+      <c r="H117" t="s">
+        <v>288</v>
+      </c>
+      <c r="I117" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J117" s="1"/>
+      <c r="M117" t="s">
+        <v>513</v>
+      </c>
+      <c r="N117" t="s">
+        <v>514</v>
+      </c>
+      <c r="O117" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>122</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="E118" t="s">
+        <v>488</v>
+      </c>
+      <c r="F118" t="s">
+        <v>20</v>
+      </c>
+      <c r="G118" t="s">
+        <v>48</v>
+      </c>
+      <c r="H118" t="s">
+        <v>288</v>
+      </c>
+      <c r="I118" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J118" s="1"/>
+      <c r="M118" t="s">
+        <v>513</v>
+      </c>
+      <c r="N118" t="s">
+        <v>514</v>
+      </c>
+      <c r="O118" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>14</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="E119" t="s">
+        <v>492</v>
+      </c>
+      <c r="G119" t="s">
+        <v>46</v>
+      </c>
+      <c r="H119" t="s">
+        <v>288</v>
+      </c>
+      <c r="I119" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J119" s="1"/>
+      <c r="M119" t="s">
+        <v>513</v>
+      </c>
+      <c r="N119" t="s">
+        <v>514</v>
+      </c>
+      <c r="O119" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>127</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="E120" t="s">
+        <v>495</v>
+      </c>
+      <c r="F120" t="s">
+        <v>1</v>
+      </c>
+      <c r="G120" t="s">
+        <v>44</v>
+      </c>
+      <c r="H120" t="s">
+        <v>288</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J120" s="1"/>
+      <c r="M120" t="s">
+        <v>513</v>
+      </c>
+      <c r="N120" t="s">
+        <v>514</v>
+      </c>
+      <c r="O120" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="E121" t="s">
+        <v>498</v>
+      </c>
+      <c r="F121" t="s">
+        <v>18</v>
+      </c>
+      <c r="G121" t="s">
+        <v>47</v>
+      </c>
+      <c r="H121" t="s">
+        <v>288</v>
+      </c>
+      <c r="I121" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J121" s="1"/>
+      <c r="M121" t="s">
+        <v>513</v>
+      </c>
+      <c r="N121" t="s">
+        <v>514</v>
+      </c>
+      <c r="O121" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>122</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="E122" t="s">
+        <v>502</v>
+      </c>
+      <c r="F122" t="s">
+        <v>20</v>
+      </c>
+      <c r="G122" t="s">
+        <v>46</v>
+      </c>
+      <c r="H122" t="s">
+        <v>288</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J122" s="1"/>
+      <c r="M122" t="s">
+        <v>513</v>
+      </c>
+      <c r="N122" t="s">
+        <v>514</v>
+      </c>
+      <c r="O122" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="E123" t="s">
+        <v>506</v>
+      </c>
+      <c r="F123" t="s">
+        <v>43</v>
+      </c>
+      <c r="G123" t="s">
+        <v>49</v>
+      </c>
+      <c r="H123" t="s">
+        <v>288</v>
+      </c>
+      <c r="I123" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J123" s="1"/>
+      <c r="M123" t="s">
+        <v>513</v>
+      </c>
+      <c r="N123" t="s">
+        <v>514</v>
+      </c>
+      <c r="O123" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>32</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="E124" t="s">
+        <v>510</v>
+      </c>
+      <c r="F124" t="s">
+        <v>511</v>
+      </c>
+      <c r="H124" t="s">
+        <v>288</v>
+      </c>
+      <c r="I124" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J124" s="1"/>
+      <c r="M124" t="s">
+        <v>513</v>
+      </c>
+      <c r="N124" t="s">
+        <v>514</v>
+      </c>
+      <c r="O124" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add events amistoso vs Bellapampa - colectivo min40 2
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cantolaoaqp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85F4F0B-EB85-4E75-A164-F1E033AD3D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C64F4A-E0A3-44EF-9D3C-304E7AAECFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5131,10 +5131,10 @@
         <v>348</v>
       </c>
       <c r="F82" t="s">
+        <v>43</v>
+      </c>
+      <c r="G82" t="s">
         <v>45</v>
-      </c>
-      <c r="G82" t="s">
-        <v>43</v>
       </c>
       <c r="H82" t="s">
         <v>288</v>

</xml_diff>

<commit_message>
eventos amistoso vs Bellapampa min40-60
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cantolaoaqp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C64F4A-E0A3-44EF-9D3C-304E7AAECFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A43785-6A3A-4B04-A5FE-2142DC160083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2117" uniqueCount="720">
   <si>
     <t>XY</t>
   </si>
@@ -1565,6 +1565,621 @@
   </si>
   <si>
     <t>True</t>
+  </si>
+  <si>
+    <t>40:54</t>
+  </si>
+  <si>
+    <t>40:57</t>
+  </si>
+  <si>
+    <t>41:01</t>
+  </si>
+  <si>
+    <t>41:27</t>
+  </si>
+  <si>
+    <t>41:32</t>
+  </si>
+  <si>
+    <t>41:36</t>
+  </si>
+  <si>
+    <t>16;90</t>
+  </si>
+  <si>
+    <t>41:59</t>
+  </si>
+  <si>
+    <t>42:16</t>
+  </si>
+  <si>
+    <t>12;16</t>
+  </si>
+  <si>
+    <t>42:20</t>
+  </si>
+  <si>
+    <t>42:25</t>
+  </si>
+  <si>
+    <t>42:30</t>
+  </si>
+  <si>
+    <t>87;8</t>
+  </si>
+  <si>
+    <t>42:28</t>
+  </si>
+  <si>
+    <t>42:34</t>
+  </si>
+  <si>
+    <t>42:40</t>
+  </si>
+  <si>
+    <t>42:51</t>
+  </si>
+  <si>
+    <t>42:56</t>
+  </si>
+  <si>
+    <t>43:01</t>
+  </si>
+  <si>
+    <t>25;14</t>
+  </si>
+  <si>
+    <t>42:58</t>
+  </si>
+  <si>
+    <t>43:04</t>
+  </si>
+  <si>
+    <t>43:11</t>
+  </si>
+  <si>
+    <t>26;66</t>
+  </si>
+  <si>
+    <t>43:59</t>
+  </si>
+  <si>
+    <t>44:06</t>
+  </si>
+  <si>
+    <t>31;31</t>
+  </si>
+  <si>
+    <t>44:03</t>
+  </si>
+  <si>
+    <t>44:10</t>
+  </si>
+  <si>
+    <t>44:17</t>
+  </si>
+  <si>
+    <t>39;41</t>
+  </si>
+  <si>
+    <t>44:12</t>
+  </si>
+  <si>
+    <t>44:22</t>
+  </si>
+  <si>
+    <t>40;16</t>
+  </si>
+  <si>
+    <t>44:32</t>
+  </si>
+  <si>
+    <t>44:36</t>
+  </si>
+  <si>
+    <t>44:40</t>
+  </si>
+  <si>
+    <t>54;23</t>
+  </si>
+  <si>
+    <t>45:17</t>
+  </si>
+  <si>
+    <t>45:20</t>
+  </si>
+  <si>
+    <t>45:24</t>
+  </si>
+  <si>
+    <t>75;62</t>
+  </si>
+  <si>
+    <t>45:39</t>
+  </si>
+  <si>
+    <t>45:44</t>
+  </si>
+  <si>
+    <t>45:48</t>
+  </si>
+  <si>
+    <t>92;91</t>
+  </si>
+  <si>
+    <t>Corner en contra</t>
+  </si>
+  <si>
+    <t>45:47</t>
+  </si>
+  <si>
+    <t>45:52</t>
+  </si>
+  <si>
+    <t>45:56</t>
+  </si>
+  <si>
+    <t>95;51</t>
+  </si>
+  <si>
+    <t>46:22</t>
+  </si>
+  <si>
+    <t>46:26</t>
+  </si>
+  <si>
+    <t>46:29</t>
+  </si>
+  <si>
+    <t>73;14</t>
+  </si>
+  <si>
+    <t>46:30</t>
+  </si>
+  <si>
+    <t>46:34</t>
+  </si>
+  <si>
+    <t>46:37</t>
+  </si>
+  <si>
+    <t>78;85</t>
+  </si>
+  <si>
+    <t>46:46</t>
+  </si>
+  <si>
+    <t>46:55</t>
+  </si>
+  <si>
+    <t>69;84</t>
+  </si>
+  <si>
+    <t>47:25</t>
+  </si>
+  <si>
+    <t>47:29</t>
+  </si>
+  <si>
+    <t>47:33</t>
+  </si>
+  <si>
+    <t>43;82</t>
+  </si>
+  <si>
+    <t>47:32</t>
+  </si>
+  <si>
+    <t>47:40</t>
+  </si>
+  <si>
+    <t>47:48</t>
+  </si>
+  <si>
+    <t>51;44</t>
+  </si>
+  <si>
+    <t>47:46</t>
+  </si>
+  <si>
+    <t>47:51</t>
+  </si>
+  <si>
+    <t>47:57</t>
+  </si>
+  <si>
+    <t>48;34</t>
+  </si>
+  <si>
+    <t>48:09</t>
+  </si>
+  <si>
+    <t>48:13</t>
+  </si>
+  <si>
+    <t>48:18</t>
+  </si>
+  <si>
+    <t>19;91</t>
+  </si>
+  <si>
+    <t>48:15</t>
+  </si>
+  <si>
+    <t>48:22</t>
+  </si>
+  <si>
+    <t>33;65</t>
+  </si>
+  <si>
+    <t>48:29</t>
+  </si>
+  <si>
+    <t>48:33</t>
+  </si>
+  <si>
+    <t>48:37</t>
+  </si>
+  <si>
+    <t>19;36</t>
+  </si>
+  <si>
+    <t>48:34</t>
+  </si>
+  <si>
+    <t>48:39</t>
+  </si>
+  <si>
+    <t>48:43</t>
+  </si>
+  <si>
+    <t>31;91</t>
+  </si>
+  <si>
+    <t>49:24</t>
+  </si>
+  <si>
+    <t>49:27</t>
+  </si>
+  <si>
+    <t>49:30</t>
+  </si>
+  <si>
+    <t>14;94</t>
+  </si>
+  <si>
+    <t>49:48</t>
+  </si>
+  <si>
+    <t>50:05</t>
+  </si>
+  <si>
+    <t>24;15</t>
+  </si>
+  <si>
+    <t>50:20</t>
+  </si>
+  <si>
+    <t>50:25</t>
+  </si>
+  <si>
+    <t>50:29</t>
+  </si>
+  <si>
+    <t>53;15</t>
+  </si>
+  <si>
+    <t>50:39</t>
+  </si>
+  <si>
+    <t>50:46</t>
+  </si>
+  <si>
+    <t>50:54</t>
+  </si>
+  <si>
+    <t>74;12</t>
+  </si>
+  <si>
+    <t>51:09</t>
+  </si>
+  <si>
+    <t>51:19</t>
+  </si>
+  <si>
+    <t>51:29</t>
+  </si>
+  <si>
+    <t>87;85</t>
+  </si>
+  <si>
+    <t>51:31</t>
+  </si>
+  <si>
+    <t>51:39</t>
+  </si>
+  <si>
+    <t>51:46</t>
+  </si>
+  <si>
+    <t>32;27</t>
+  </si>
+  <si>
+    <t>51:54</t>
+  </si>
+  <si>
+    <t>51:59</t>
+  </si>
+  <si>
+    <t>52:03</t>
+  </si>
+  <si>
+    <t>16;73</t>
+  </si>
+  <si>
+    <t>53:22</t>
+  </si>
+  <si>
+    <t>53:28</t>
+  </si>
+  <si>
+    <t>53:34</t>
+  </si>
+  <si>
+    <t>67;27</t>
+  </si>
+  <si>
+    <t>54:14</t>
+  </si>
+  <si>
+    <t>54:19</t>
+  </si>
+  <si>
+    <t>54:25</t>
+  </si>
+  <si>
+    <t>30;52</t>
+  </si>
+  <si>
+    <t>54:47</t>
+  </si>
+  <si>
+    <t>54:49</t>
+  </si>
+  <si>
+    <t>54:52</t>
+  </si>
+  <si>
+    <t>23;60</t>
+  </si>
+  <si>
+    <t>54:51</t>
+  </si>
+  <si>
+    <t>54:54</t>
+  </si>
+  <si>
+    <t>54:57</t>
+  </si>
+  <si>
+    <t>25;81</t>
+  </si>
+  <si>
+    <t>55:18</t>
+  </si>
+  <si>
+    <t>55:24</t>
+  </si>
+  <si>
+    <t>55:30</t>
+  </si>
+  <si>
+    <t>9;61</t>
+  </si>
+  <si>
+    <t>55:31</t>
+  </si>
+  <si>
+    <t>55:35</t>
+  </si>
+  <si>
+    <t>55:39</t>
+  </si>
+  <si>
+    <t>60;32</t>
+  </si>
+  <si>
+    <t>55:43</t>
+  </si>
+  <si>
+    <t>55:48</t>
+  </si>
+  <si>
+    <t>92;47</t>
+  </si>
+  <si>
+    <t>55:45</t>
+  </si>
+  <si>
+    <t>55:51</t>
+  </si>
+  <si>
+    <t>55:57</t>
+  </si>
+  <si>
+    <t>68;23</t>
+  </si>
+  <si>
+    <t>56:17</t>
+  </si>
+  <si>
+    <t>56:29</t>
+  </si>
+  <si>
+    <t>56:40</t>
+  </si>
+  <si>
+    <t>91;35</t>
+  </si>
+  <si>
+    <t>57:13</t>
+  </si>
+  <si>
+    <t>57:17</t>
+  </si>
+  <si>
+    <t>57:22</t>
+  </si>
+  <si>
+    <t>8;86</t>
+  </si>
+  <si>
+    <t>57:27</t>
+  </si>
+  <si>
+    <t>57:31</t>
+  </si>
+  <si>
+    <t>57:35</t>
+  </si>
+  <si>
+    <t>6;47</t>
+  </si>
+  <si>
+    <t>57:39</t>
+  </si>
+  <si>
+    <t>57:44</t>
+  </si>
+  <si>
+    <t>32;22</t>
+  </si>
+  <si>
+    <t>57:52</t>
+  </si>
+  <si>
+    <t>57:58</t>
+  </si>
+  <si>
+    <t>58:03</t>
+  </si>
+  <si>
+    <t>20;92</t>
+  </si>
+  <si>
+    <t>58:12</t>
+  </si>
+  <si>
+    <t>58:17</t>
+  </si>
+  <si>
+    <t>58:22</t>
+  </si>
+  <si>
+    <t>67;79</t>
+  </si>
+  <si>
+    <t>59:01</t>
+  </si>
+  <si>
+    <t>59:11</t>
+  </si>
+  <si>
+    <t>59:20</t>
+  </si>
+  <si>
+    <t>60:07</t>
+  </si>
+  <si>
+    <t>60:22</t>
+  </si>
+  <si>
+    <t>60:37</t>
+  </si>
+  <si>
+    <t>41;66</t>
+  </si>
+  <si>
+    <t>60:35</t>
+  </si>
+  <si>
+    <t>60:40</t>
+  </si>
+  <si>
+    <t>60:45</t>
+  </si>
+  <si>
+    <t>19;10</t>
+  </si>
+  <si>
+    <t>60:48</t>
+  </si>
+  <si>
+    <t>60:52</t>
+  </si>
+  <si>
+    <t>13;86</t>
+  </si>
+  <si>
+    <t>60:51</t>
+  </si>
+  <si>
+    <t>60:56</t>
+  </si>
+  <si>
+    <t>61:00</t>
+  </si>
+  <si>
+    <t>32;74</t>
+  </si>
+  <si>
+    <t>61:04</t>
+  </si>
+  <si>
+    <t>61:08</t>
+  </si>
+  <si>
+    <t>61:12</t>
+  </si>
+  <si>
+    <t>39;49</t>
+  </si>
+  <si>
+    <t>61:11</t>
+  </si>
+  <si>
+    <t>61:14</t>
+  </si>
+  <si>
+    <t>61:17</t>
+  </si>
+  <si>
+    <t>68;53</t>
+  </si>
+  <si>
+    <t>61:16</t>
+  </si>
+  <si>
+    <t>61:20</t>
+  </si>
+  <si>
+    <t>61:24</t>
+  </si>
+  <si>
+    <t>49;60</t>
+  </si>
+  <si>
+    <t>61:21</t>
+  </si>
+  <si>
+    <t>61:26</t>
+  </si>
+  <si>
+    <t>61:32</t>
+  </si>
+  <si>
+    <t>43;74</t>
   </si>
 </sst>
 </file>
@@ -1647,8 +2262,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}" name="Tabla1" displayName="Tabla1" ref="A1:O124" totalsRowShown="0">
-  <autoFilter ref="A1:O124" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}" name="Tabla1" displayName="Tabla1" ref="A1:O178" totalsRowShown="0">
+  <autoFilter ref="A1:O178" xr:uid="{C1975CA6-E80E-40A4-A9D5-728F867A63BD}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{45CCCD5A-AFCF-487D-ADA1-0BFBB6505772}" name="Event"/>
     <tableColumn id="2" xr3:uid="{4A939A0F-B787-4665-B94F-35DE80E0B243}" name="start_time" dataDxfId="2"/>
@@ -1957,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77939FC4-FC73-4262-977F-310955BE7B1D}">
-  <dimension ref="A1:O124"/>
+  <dimension ref="A1:O178"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5703125" customWidth="1"/>
@@ -6764,6 +7379,2097 @@
         <v>55</v>
       </c>
     </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>127</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="E125" t="s">
+        <v>245</v>
+      </c>
+      <c r="F125" t="s">
+        <v>43</v>
+      </c>
+      <c r="G125" t="s">
+        <v>44</v>
+      </c>
+      <c r="H125" t="s">
+        <v>288</v>
+      </c>
+      <c r="I125" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J125" s="1"/>
+      <c r="M125" t="s">
+        <v>513</v>
+      </c>
+      <c r="N125" t="s">
+        <v>514</v>
+      </c>
+      <c r="O125" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>32</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="E126" t="s">
+        <v>521</v>
+      </c>
+      <c r="F126" t="s">
+        <v>4</v>
+      </c>
+      <c r="G126" t="s">
+        <v>49</v>
+      </c>
+      <c r="H126" t="s">
+        <v>288</v>
+      </c>
+      <c r="I126" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J126" s="1"/>
+      <c r="M126" t="s">
+        <v>513</v>
+      </c>
+      <c r="N126" t="s">
+        <v>514</v>
+      </c>
+      <c r="O126" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>14</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="E127" t="s">
+        <v>524</v>
+      </c>
+      <c r="F127" t="s">
+        <v>42</v>
+      </c>
+      <c r="G127" t="s">
+        <v>287</v>
+      </c>
+      <c r="H127" t="s">
+        <v>288</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J127" s="1"/>
+      <c r="M127" t="s">
+        <v>513</v>
+      </c>
+      <c r="N127" t="s">
+        <v>514</v>
+      </c>
+      <c r="O127" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>14</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="E128" t="s">
+        <v>528</v>
+      </c>
+      <c r="F128" t="s">
+        <v>20</v>
+      </c>
+      <c r="G128" t="s">
+        <v>46</v>
+      </c>
+      <c r="H128" t="s">
+        <v>288</v>
+      </c>
+      <c r="I128" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J128" s="1"/>
+      <c r="M128" t="s">
+        <v>513</v>
+      </c>
+      <c r="N128" t="s">
+        <v>514</v>
+      </c>
+      <c r="O128" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>127</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="E129" t="s">
+        <v>402</v>
+      </c>
+      <c r="F129" t="s">
+        <v>43</v>
+      </c>
+      <c r="G129" t="s">
+        <v>45</v>
+      </c>
+      <c r="H129" t="s">
+        <v>288</v>
+      </c>
+      <c r="I129" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J129" s="1"/>
+      <c r="M129" t="s">
+        <v>513</v>
+      </c>
+      <c r="N129" t="s">
+        <v>514</v>
+      </c>
+      <c r="O129" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>14</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="E130" t="s">
+        <v>535</v>
+      </c>
+      <c r="F130" t="s">
+        <v>20</v>
+      </c>
+      <c r="G130" t="s">
+        <v>287</v>
+      </c>
+      <c r="H130" t="s">
+        <v>288</v>
+      </c>
+      <c r="I130" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J130" s="1"/>
+      <c r="M130" t="s">
+        <v>513</v>
+      </c>
+      <c r="N130" t="s">
+        <v>514</v>
+      </c>
+      <c r="O130" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>127</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="E131" t="s">
+        <v>539</v>
+      </c>
+      <c r="F131" t="s">
+        <v>43</v>
+      </c>
+      <c r="G131" t="s">
+        <v>49</v>
+      </c>
+      <c r="H131" t="s">
+        <v>288</v>
+      </c>
+      <c r="I131" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J131" s="1"/>
+      <c r="L131" t="s">
+        <v>512</v>
+      </c>
+      <c r="M131" t="s">
+        <v>513</v>
+      </c>
+      <c r="N131" t="s">
+        <v>514</v>
+      </c>
+      <c r="O131" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>14</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E132" t="s">
+        <v>542</v>
+      </c>
+      <c r="F132" t="s">
+        <v>20</v>
+      </c>
+      <c r="G132" t="s">
+        <v>46</v>
+      </c>
+      <c r="H132" t="s">
+        <v>288</v>
+      </c>
+      <c r="I132" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J132" s="1"/>
+      <c r="M132" t="s">
+        <v>513</v>
+      </c>
+      <c r="N132" t="s">
+        <v>514</v>
+      </c>
+      <c r="O132" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>127</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E133" t="s">
+        <v>546</v>
+      </c>
+      <c r="F133" t="s">
+        <v>1</v>
+      </c>
+      <c r="G133" t="s">
+        <v>47</v>
+      </c>
+      <c r="H133" t="s">
+        <v>288</v>
+      </c>
+      <c r="I133" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J133" s="1"/>
+      <c r="M133" t="s">
+        <v>513</v>
+      </c>
+      <c r="N133" t="s">
+        <v>514</v>
+      </c>
+      <c r="O133" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>122</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="E134" t="s">
+        <v>549</v>
+      </c>
+      <c r="F134" t="s">
+        <v>20</v>
+      </c>
+      <c r="G134" t="s">
+        <v>48</v>
+      </c>
+      <c r="H134" t="s">
+        <v>288</v>
+      </c>
+      <c r="I134" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J134" s="1"/>
+      <c r="M134" t="s">
+        <v>513</v>
+      </c>
+      <c r="N134" t="s">
+        <v>514</v>
+      </c>
+      <c r="O134" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
+        <v>27</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="E135" t="s">
+        <v>553</v>
+      </c>
+      <c r="F135" t="s">
+        <v>15</v>
+      </c>
+      <c r="H135" t="s">
+        <v>288</v>
+      </c>
+      <c r="I135" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J135" s="1"/>
+      <c r="M135" t="s">
+        <v>513</v>
+      </c>
+      <c r="N135" t="s">
+        <v>514</v>
+      </c>
+      <c r="O135" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>27</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="E136" t="s">
+        <v>557</v>
+      </c>
+      <c r="F136" t="s">
+        <v>15</v>
+      </c>
+      <c r="G136" t="s">
+        <v>49</v>
+      </c>
+      <c r="H136" t="s">
+        <v>288</v>
+      </c>
+      <c r="I136" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J136" s="1"/>
+      <c r="M136" t="s">
+        <v>513</v>
+      </c>
+      <c r="N136" t="s">
+        <v>514</v>
+      </c>
+      <c r="O136" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
+        <v>27</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="E137" t="s">
+        <v>561</v>
+      </c>
+      <c r="F137" t="s">
+        <v>562</v>
+      </c>
+      <c r="H137" t="s">
+        <v>288</v>
+      </c>
+      <c r="I137" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J137" s="1"/>
+      <c r="M137" t="s">
+        <v>513</v>
+      </c>
+      <c r="N137" t="s">
+        <v>514</v>
+      </c>
+      <c r="O137" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>127</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="E138" t="s">
+        <v>566</v>
+      </c>
+      <c r="F138" t="s">
+        <v>43</v>
+      </c>
+      <c r="G138" t="s">
+        <v>47</v>
+      </c>
+      <c r="H138" t="s">
+        <v>288</v>
+      </c>
+      <c r="I138" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J138" s="1"/>
+      <c r="M138" t="s">
+        <v>513</v>
+      </c>
+      <c r="N138" t="s">
+        <v>514</v>
+      </c>
+      <c r="O138" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
+        <v>27</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="E139" t="s">
+        <v>570</v>
+      </c>
+      <c r="F139" t="s">
+        <v>15</v>
+      </c>
+      <c r="H139" t="s">
+        <v>288</v>
+      </c>
+      <c r="I139" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J139" s="1"/>
+      <c r="M139" t="s">
+        <v>513</v>
+      </c>
+      <c r="N139" t="s">
+        <v>514</v>
+      </c>
+      <c r="O139" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>127</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="E140" t="s">
+        <v>574</v>
+      </c>
+      <c r="F140" t="s">
+        <v>43</v>
+      </c>
+      <c r="G140" t="s">
+        <v>44</v>
+      </c>
+      <c r="H140" t="s">
+        <v>288</v>
+      </c>
+      <c r="I140" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J140" s="1"/>
+      <c r="M140" t="s">
+        <v>513</v>
+      </c>
+      <c r="N140" t="s">
+        <v>514</v>
+      </c>
+      <c r="O140" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
+        <v>2</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="E141" t="s">
+        <v>577</v>
+      </c>
+      <c r="F141" t="s">
+        <v>17</v>
+      </c>
+      <c r="G141" t="s">
+        <v>47</v>
+      </c>
+      <c r="H141" t="s">
+        <v>288</v>
+      </c>
+      <c r="I141" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J141" s="1"/>
+      <c r="M141" t="s">
+        <v>513</v>
+      </c>
+      <c r="N141" t="s">
+        <v>514</v>
+      </c>
+      <c r="O141" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
+        <v>127</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="E142" t="s">
+        <v>581</v>
+      </c>
+      <c r="F142" t="s">
+        <v>1</v>
+      </c>
+      <c r="G142" t="s">
+        <v>47</v>
+      </c>
+      <c r="H142" t="s">
+        <v>288</v>
+      </c>
+      <c r="I142" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J142" s="1"/>
+      <c r="M142" t="s">
+        <v>513</v>
+      </c>
+      <c r="N142" t="s">
+        <v>514</v>
+      </c>
+      <c r="O142" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>122</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="E143" t="s">
+        <v>585</v>
+      </c>
+      <c r="F143" t="s">
+        <v>20</v>
+      </c>
+      <c r="G143" t="s">
+        <v>46</v>
+      </c>
+      <c r="H143" t="s">
+        <v>288</v>
+      </c>
+      <c r="I143" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J143" s="1"/>
+      <c r="M143" t="s">
+        <v>513</v>
+      </c>
+      <c r="N143" t="s">
+        <v>514</v>
+      </c>
+      <c r="O143" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>127</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="E144" t="s">
+        <v>589</v>
+      </c>
+      <c r="F144" t="s">
+        <v>43</v>
+      </c>
+      <c r="G144" t="s">
+        <v>47</v>
+      </c>
+      <c r="H144" t="s">
+        <v>288</v>
+      </c>
+      <c r="I144" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J144" s="1"/>
+      <c r="M144" t="s">
+        <v>513</v>
+      </c>
+      <c r="N144" t="s">
+        <v>514</v>
+      </c>
+      <c r="O144" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>14</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="E145" t="s">
+        <v>593</v>
+      </c>
+      <c r="F145" t="s">
+        <v>20</v>
+      </c>
+      <c r="G145" t="s">
+        <v>46</v>
+      </c>
+      <c r="H145" t="s">
+        <v>288</v>
+      </c>
+      <c r="I145" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J145" s="1"/>
+      <c r="M145" t="s">
+        <v>513</v>
+      </c>
+      <c r="N145" t="s">
+        <v>514</v>
+      </c>
+      <c r="O145" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>127</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="E146" t="s">
+        <v>596</v>
+      </c>
+      <c r="F146" t="s">
+        <v>43</v>
+      </c>
+      <c r="G146" t="s">
+        <v>47</v>
+      </c>
+      <c r="H146" t="s">
+        <v>288</v>
+      </c>
+      <c r="I146" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J146" s="1"/>
+      <c r="M146" t="s">
+        <v>513</v>
+      </c>
+      <c r="N146" t="s">
+        <v>514</v>
+      </c>
+      <c r="O146" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
+        <v>14</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="E147" t="s">
+        <v>600</v>
+      </c>
+      <c r="F147" t="s">
+        <v>42</v>
+      </c>
+      <c r="G147" t="s">
+        <v>46</v>
+      </c>
+      <c r="H147" t="s">
+        <v>288</v>
+      </c>
+      <c r="I147" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J147" s="1"/>
+      <c r="M147" t="s">
+        <v>513</v>
+      </c>
+      <c r="N147" t="s">
+        <v>514</v>
+      </c>
+      <c r="O147" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
+        <v>127</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="E148" t="s">
+        <v>604</v>
+      </c>
+      <c r="F148" t="s">
+        <v>43</v>
+      </c>
+      <c r="G148" t="s">
+        <v>44</v>
+      </c>
+      <c r="H148" t="s">
+        <v>288</v>
+      </c>
+      <c r="I148" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J148" s="1"/>
+      <c r="M148" t="s">
+        <v>513</v>
+      </c>
+      <c r="N148" t="s">
+        <v>514</v>
+      </c>
+      <c r="O148" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
+        <v>32</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>605</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="E149" t="s">
+        <v>608</v>
+      </c>
+      <c r="F149" t="s">
+        <v>4</v>
+      </c>
+      <c r="H149" t="s">
+        <v>288</v>
+      </c>
+      <c r="I149" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J149" s="1"/>
+      <c r="M149" t="s">
+        <v>513</v>
+      </c>
+      <c r="N149" t="s">
+        <v>514</v>
+      </c>
+      <c r="O149" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>14</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="E150" t="s">
+        <v>611</v>
+      </c>
+      <c r="F150" t="s">
+        <v>20</v>
+      </c>
+      <c r="G150" t="s">
+        <v>287</v>
+      </c>
+      <c r="H150" t="s">
+        <v>288</v>
+      </c>
+      <c r="I150" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J150" s="1"/>
+      <c r="M150" t="s">
+        <v>513</v>
+      </c>
+      <c r="N150" t="s">
+        <v>514</v>
+      </c>
+      <c r="O150" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>27</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="E151" t="s">
+        <v>615</v>
+      </c>
+      <c r="F151" t="s">
+        <v>15</v>
+      </c>
+      <c r="H151" t="s">
+        <v>288</v>
+      </c>
+      <c r="I151" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J151" s="1"/>
+      <c r="M151" t="s">
+        <v>513</v>
+      </c>
+      <c r="N151" t="s">
+        <v>514</v>
+      </c>
+      <c r="O151" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>14</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="E152" t="s">
+        <v>619</v>
+      </c>
+      <c r="F152" t="s">
+        <v>20</v>
+      </c>
+      <c r="G152" t="s">
+        <v>48</v>
+      </c>
+      <c r="H152" t="s">
+        <v>288</v>
+      </c>
+      <c r="I152" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J152" s="1"/>
+      <c r="M152" t="s">
+        <v>513</v>
+      </c>
+      <c r="N152" t="s">
+        <v>514</v>
+      </c>
+      <c r="O152" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>127</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="E153" t="s">
+        <v>623</v>
+      </c>
+      <c r="F153" t="s">
+        <v>43</v>
+      </c>
+      <c r="G153" t="s">
+        <v>45</v>
+      </c>
+      <c r="H153" t="s">
+        <v>288</v>
+      </c>
+      <c r="I153" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J153" s="1"/>
+      <c r="M153" t="s">
+        <v>513</v>
+      </c>
+      <c r="N153" t="s">
+        <v>514</v>
+      </c>
+      <c r="O153" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="154" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
+        <v>127</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="E154" t="s">
+        <v>627</v>
+      </c>
+      <c r="F154" t="s">
+        <v>43</v>
+      </c>
+      <c r="G154" t="s">
+        <v>49</v>
+      </c>
+      <c r="H154" t="s">
+        <v>288</v>
+      </c>
+      <c r="I154" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J154" s="1"/>
+      <c r="M154" t="s">
+        <v>513</v>
+      </c>
+      <c r="N154" t="s">
+        <v>514</v>
+      </c>
+      <c r="O154" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="155" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>14</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="C155" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="E155" t="s">
+        <v>631</v>
+      </c>
+      <c r="F155" t="s">
+        <v>20</v>
+      </c>
+      <c r="G155" t="s">
+        <v>48</v>
+      </c>
+      <c r="H155" t="s">
+        <v>288</v>
+      </c>
+      <c r="I155" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J155" s="1"/>
+      <c r="M155" t="s">
+        <v>513</v>
+      </c>
+      <c r="N155" t="s">
+        <v>514</v>
+      </c>
+      <c r="O155" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="156" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="E156" t="s">
+        <v>635</v>
+      </c>
+      <c r="F156" t="s">
+        <v>3</v>
+      </c>
+      <c r="G156" t="s">
+        <v>44</v>
+      </c>
+      <c r="H156" t="s">
+        <v>288</v>
+      </c>
+      <c r="I156" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J156" s="1"/>
+      <c r="M156" t="s">
+        <v>513</v>
+      </c>
+      <c r="N156" t="s">
+        <v>514</v>
+      </c>
+      <c r="O156" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
+        <v>32</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="E157" t="s">
+        <v>639</v>
+      </c>
+      <c r="F157" t="s">
+        <v>4</v>
+      </c>
+      <c r="G157" t="s">
+        <v>49</v>
+      </c>
+      <c r="H157" t="s">
+        <v>288</v>
+      </c>
+      <c r="I157" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J157" s="1"/>
+      <c r="M157" t="s">
+        <v>513</v>
+      </c>
+      <c r="N157" t="s">
+        <v>514</v>
+      </c>
+      <c r="O157" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="158" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
+        <v>14</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="E158" t="s">
+        <v>643</v>
+      </c>
+      <c r="F158" t="s">
+        <v>20</v>
+      </c>
+      <c r="G158" t="s">
+        <v>46</v>
+      </c>
+      <c r="H158" t="s">
+        <v>288</v>
+      </c>
+      <c r="I158" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J158" s="1"/>
+      <c r="M158" t="s">
+        <v>513</v>
+      </c>
+      <c r="N158" t="s">
+        <v>514</v>
+      </c>
+      <c r="O158" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
+        <v>127</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="E159" t="s">
+        <v>647</v>
+      </c>
+      <c r="F159" t="s">
+        <v>43</v>
+      </c>
+      <c r="G159" t="s">
+        <v>44</v>
+      </c>
+      <c r="H159" t="s">
+        <v>288</v>
+      </c>
+      <c r="I159" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J159" s="1"/>
+      <c r="M159" t="s">
+        <v>513</v>
+      </c>
+      <c r="N159" t="s">
+        <v>514</v>
+      </c>
+      <c r="O159" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="160" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
+        <v>32</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="E160" t="s">
+        <v>651</v>
+      </c>
+      <c r="F160" t="s">
+        <v>511</v>
+      </c>
+      <c r="H160" t="s">
+        <v>288</v>
+      </c>
+      <c r="I160" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J160" s="1"/>
+      <c r="M160" t="s">
+        <v>513</v>
+      </c>
+      <c r="N160" t="s">
+        <v>514</v>
+      </c>
+      <c r="O160" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="161" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
+        <v>14</v>
+      </c>
+      <c r="B161" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="E161" t="s">
+        <v>655</v>
+      </c>
+      <c r="G161" t="s">
+        <v>46</v>
+      </c>
+      <c r="H161" t="s">
+        <v>288</v>
+      </c>
+      <c r="I161" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J161" s="1"/>
+      <c r="M161" t="s">
+        <v>513</v>
+      </c>
+      <c r="N161" t="s">
+        <v>514</v>
+      </c>
+      <c r="O161" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="162" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
+        <v>127</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="E162" t="s">
+        <v>658</v>
+      </c>
+      <c r="F162" t="s">
+        <v>43</v>
+      </c>
+      <c r="G162" t="s">
+        <v>47</v>
+      </c>
+      <c r="H162" t="s">
+        <v>288</v>
+      </c>
+      <c r="I162" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J162" s="1"/>
+      <c r="M162" t="s">
+        <v>513</v>
+      </c>
+      <c r="N162" t="s">
+        <v>514</v>
+      </c>
+      <c r="O162" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="163" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
+        <v>122</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="E163" t="s">
+        <v>662</v>
+      </c>
+      <c r="F163" t="s">
+        <v>20</v>
+      </c>
+      <c r="G163" t="s">
+        <v>419</v>
+      </c>
+      <c r="H163" t="s">
+        <v>288</v>
+      </c>
+      <c r="I163" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J163" s="1"/>
+      <c r="M163" t="s">
+        <v>513</v>
+      </c>
+      <c r="N163" t="s">
+        <v>514</v>
+      </c>
+      <c r="O163" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="164" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
+        <v>2</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="E164" t="s">
+        <v>666</v>
+      </c>
+      <c r="F164" t="s">
+        <v>17</v>
+      </c>
+      <c r="G164" t="s">
+        <v>45</v>
+      </c>
+      <c r="H164" t="s">
+        <v>288</v>
+      </c>
+      <c r="I164" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J164" s="1"/>
+      <c r="M164" t="s">
+        <v>513</v>
+      </c>
+      <c r="N164" t="s">
+        <v>514</v>
+      </c>
+      <c r="O164" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="165" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
+        <v>32</v>
+      </c>
+      <c r="B165" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="C165" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="D165" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="E165" t="s">
+        <v>670</v>
+      </c>
+      <c r="F165" t="s">
+        <v>4</v>
+      </c>
+      <c r="G165" t="s">
+        <v>49</v>
+      </c>
+      <c r="H165" t="s">
+        <v>288</v>
+      </c>
+      <c r="I165" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J165" s="1"/>
+      <c r="M165" t="s">
+        <v>513</v>
+      </c>
+      <c r="N165" t="s">
+        <v>514</v>
+      </c>
+      <c r="O165" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="166" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
+        <v>122</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>673</v>
+      </c>
+      <c r="E166" t="s">
+        <v>674</v>
+      </c>
+      <c r="F166" t="s">
+        <v>21</v>
+      </c>
+      <c r="G166" t="s">
+        <v>46</v>
+      </c>
+      <c r="H166" t="s">
+        <v>288</v>
+      </c>
+      <c r="I166" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J166" s="1"/>
+      <c r="M166" t="s">
+        <v>513</v>
+      </c>
+      <c r="N166" t="s">
+        <v>514</v>
+      </c>
+      <c r="O166" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="167" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A167" t="s">
+        <v>127</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>673</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="E167" t="s">
+        <v>677</v>
+      </c>
+      <c r="F167" t="s">
+        <v>43</v>
+      </c>
+      <c r="G167" t="s">
+        <v>47</v>
+      </c>
+      <c r="H167" t="s">
+        <v>288</v>
+      </c>
+      <c r="I167" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J167" s="1"/>
+      <c r="M167" t="s">
+        <v>513</v>
+      </c>
+      <c r="N167" t="s">
+        <v>514</v>
+      </c>
+      <c r="O167" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="168" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A168" t="s">
+        <v>14</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="E168" t="s">
+        <v>681</v>
+      </c>
+      <c r="F168" t="s">
+        <v>20</v>
+      </c>
+      <c r="G168" t="s">
+        <v>48</v>
+      </c>
+      <c r="H168" t="s">
+        <v>288</v>
+      </c>
+      <c r="I168" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J168" s="1"/>
+      <c r="M168" t="s">
+        <v>513</v>
+      </c>
+      <c r="N168" t="s">
+        <v>514</v>
+      </c>
+      <c r="O168" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="169" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A169" t="s">
+        <v>14</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="C169" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="D169" s="3" t="s">
+        <v>684</v>
+      </c>
+      <c r="E169" t="s">
+        <v>685</v>
+      </c>
+      <c r="F169" t="s">
+        <v>42</v>
+      </c>
+      <c r="G169" t="s">
+        <v>287</v>
+      </c>
+      <c r="H169" t="s">
+        <v>288</v>
+      </c>
+      <c r="I169" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J169" s="1"/>
+      <c r="M169" t="s">
+        <v>513</v>
+      </c>
+      <c r="N169" t="s">
+        <v>514</v>
+      </c>
+      <c r="O169" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="170" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A170" t="s">
+        <v>2</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D170" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="E170" t="s">
+        <v>566</v>
+      </c>
+      <c r="F170" t="s">
+        <v>17</v>
+      </c>
+      <c r="G170" t="s">
+        <v>49</v>
+      </c>
+      <c r="H170" t="s">
+        <v>288</v>
+      </c>
+      <c r="I170" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J170" s="1"/>
+      <c r="L170" t="s">
+        <v>512</v>
+      </c>
+      <c r="M170" t="s">
+        <v>513</v>
+      </c>
+      <c r="N170" t="s">
+        <v>514</v>
+      </c>
+      <c r="O170" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="171" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A171" t="s">
+        <v>14</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="C171" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="D171" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="E171" t="s">
+        <v>692</v>
+      </c>
+      <c r="F171" t="s">
+        <v>20</v>
+      </c>
+      <c r="G171" t="s">
+        <v>46</v>
+      </c>
+      <c r="H171" t="s">
+        <v>288</v>
+      </c>
+      <c r="I171" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J171" s="1"/>
+      <c r="M171" t="s">
+        <v>513</v>
+      </c>
+      <c r="N171" t="s">
+        <v>514</v>
+      </c>
+      <c r="O171" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="172" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A172" t="s">
+        <v>127</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="C172" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="E172" t="s">
+        <v>696</v>
+      </c>
+      <c r="F172" t="s">
+        <v>43</v>
+      </c>
+      <c r="G172" t="s">
+        <v>49</v>
+      </c>
+      <c r="H172" t="s">
+        <v>288</v>
+      </c>
+      <c r="I172" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J172" s="1"/>
+      <c r="M172" t="s">
+        <v>513</v>
+      </c>
+      <c r="N172" t="s">
+        <v>514</v>
+      </c>
+      <c r="O172" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="173" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A173" t="s">
+        <v>122</v>
+      </c>
+      <c r="B173" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="D173" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="E173" t="s">
+        <v>699</v>
+      </c>
+      <c r="F173" t="s">
+        <v>20</v>
+      </c>
+      <c r="G173" t="s">
+        <v>46</v>
+      </c>
+      <c r="H173" t="s">
+        <v>288</v>
+      </c>
+      <c r="I173" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J173" s="1"/>
+      <c r="M173" t="s">
+        <v>513</v>
+      </c>
+      <c r="N173" t="s">
+        <v>514</v>
+      </c>
+      <c r="O173" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="174" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A174" t="s">
+        <v>2</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="C174" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D174" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="E174" t="s">
+        <v>703</v>
+      </c>
+      <c r="F174" t="s">
+        <v>17</v>
+      </c>
+      <c r="G174" t="s">
+        <v>47</v>
+      </c>
+      <c r="H174" t="s">
+        <v>288</v>
+      </c>
+      <c r="I174" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J174" s="1"/>
+      <c r="M174" t="s">
+        <v>513</v>
+      </c>
+      <c r="N174" t="s">
+        <v>514</v>
+      </c>
+      <c r="O174" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="175" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A175" t="s">
+        <v>122</v>
+      </c>
+      <c r="B175" s="3" t="s">
+        <v>704</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="D175" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="E175" t="s">
+        <v>707</v>
+      </c>
+      <c r="F175" t="s">
+        <v>20</v>
+      </c>
+      <c r="G175" t="s">
+        <v>46</v>
+      </c>
+      <c r="H175" t="s">
+        <v>288</v>
+      </c>
+      <c r="I175" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J175" s="1"/>
+      <c r="M175" t="s">
+        <v>513</v>
+      </c>
+      <c r="N175" t="s">
+        <v>514</v>
+      </c>
+      <c r="O175" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="176" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A176" t="s">
+        <v>127</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="E176" t="s">
+        <v>711</v>
+      </c>
+      <c r="F176" t="s">
+        <v>43</v>
+      </c>
+      <c r="G176" t="s">
+        <v>47</v>
+      </c>
+      <c r="H176" t="s">
+        <v>288</v>
+      </c>
+      <c r="I176" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J176" s="1"/>
+      <c r="M176" t="s">
+        <v>513</v>
+      </c>
+      <c r="N176" t="s">
+        <v>514</v>
+      </c>
+      <c r="O176" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="177" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A177" t="s">
+        <v>122</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="D177" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="E177" t="s">
+        <v>715</v>
+      </c>
+      <c r="F177" t="s">
+        <v>20</v>
+      </c>
+      <c r="G177" t="s">
+        <v>46</v>
+      </c>
+      <c r="H177" t="s">
+        <v>288</v>
+      </c>
+      <c r="I177" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J177" s="1"/>
+      <c r="M177" t="s">
+        <v>513</v>
+      </c>
+      <c r="N177" t="s">
+        <v>514</v>
+      </c>
+      <c r="O177" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="178" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A178" t="s">
+        <v>127</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>716</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="D178" s="3" t="s">
+        <v>718</v>
+      </c>
+      <c r="E178" t="s">
+        <v>719</v>
+      </c>
+      <c r="F178" t="s">
+        <v>43</v>
+      </c>
+      <c r="G178" t="s">
+        <v>44</v>
+      </c>
+      <c r="H178" t="s">
+        <v>288</v>
+      </c>
+      <c r="I178" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J178" s="1"/>
+      <c r="M178" t="s">
+        <v>513</v>
+      </c>
+      <c r="N178" t="s">
+        <v>514</v>
+      </c>
+      <c r="O178" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
eventos amistoso vs Bellapampa min40-60 corregir
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cantolaoaqp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A43785-6A3A-4B04-A5FE-2142DC160083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8B8E58-C77E-4E4B-BB47-30AA183E9FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7828,7 +7828,7 @@
         <v>15</v>
       </c>
       <c r="G136" t="s">
-        <v>49</v>
+        <v>419</v>
       </c>
       <c r="H136" t="s">
         <v>288</v>

</xml_diff>